<commit_message>
Refactor Flask API for WordPress landing page generation; consolidate helper functions, remove deprecated files, and enhance error handling. Update configuration for WordPress publishing and streamline Excel/CSV processing.
</commit_message>
<xml_diff>
--- a/bulk_upload_template.xlsx
+++ b/bulk_upload_template.xlsx
@@ -1,43 +1,89 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Last_wordpress\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35456654-077C-48BA-98AE-69B9F6E7DA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+  <si>
+    <t>sales_page_url</t>
+  </si>
+  <si>
+    <t>jv_doc_url</t>
+  </si>
+  <si>
+    <t>affiliate_link</t>
+  </si>
+  <si>
+    <t>wordpress_page_title</t>
+  </si>
+  <si>
+    <t>https://warriorplus.com/o2/link1</t>
+  </si>
+  <si>
+    <t>Hero_image</t>
+  </si>
+  <si>
+    <t>https://www.ketoflow.app/ketoflow-uploads/d6b7ff8f-4055-4818-b642-35baef0b55f3.png</t>
+  </si>
+  <si>
+    <t>https://getagentx.com/order/</t>
+  </si>
+  <si>
+    <t>Special Offer For TODAY ONLY (Profit With 25,500 AI Bots... If You Act TODAY!</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -46,93 +92,60 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,99 +433,51 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" customWidth="1"/>
+    <col min="3" max="4" width="30.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>sales_page_url</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>jv_doc_url</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>affiliate_link</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>wordpress_page_title</t>
-        </is>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>https://www.ketoflow.app/d</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://example.com/jv1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>https://warriorplus.com/o2/link1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>KetoFlow Review - Weight Loss</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>https://www.example.com/product2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>https://example.com/affiliate2</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Product Two Review</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>https://www.example.com/product3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://example.com/jv3</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>https://example.com/affiliate3</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Product Three Review</t>
-        </is>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{3F5645DE-D60D-4810-A058-FF51F185C5D1}"/>
+    <hyperlink ref="E2" r:id="rId2" xr:uid="{4A44B6D6-0773-486B-8E4C-C13673DB5957}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor price scraper agent to v3: Enhance extraction pipeline with multi-strategy approach, improve regex and DOM extraction, and update AI interpretation for better accuracy. Update CSS styles in Elementor landing builder for improved design consistency and readability. Modify bulk upload template for better data handling.
</commit_message>
<xml_diff>
--- a/bulk_upload_template.xlsx
+++ b/bulk_upload_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Last_wordpress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35456654-077C-48BA-98AE-69B9F6E7DA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{700D0DD2-A3F5-4AF5-A42E-527FAD135145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="17">
   <si>
     <t>sales_page_url</t>
   </si>
@@ -43,17 +43,43 @@
     <t>https://www.ketoflow.app/ketoflow-uploads/d6b7ff8f-4055-4818-b642-35baef0b55f3.png</t>
   </si>
   <si>
+    <t>Special Offer For TODAY ONLY (Profit With 25,500 AI Bots... If You Act TODAY!</t>
+  </si>
+  <si>
     <t>https://getagentx.com/order/</t>
   </si>
   <si>
-    <t>Special Offer For TODAY ONLY (Profit With 25,500 AI Bots... If You Act TODAY!</t>
+    <t>https://www.ketoflow.app/d</t>
+  </si>
+  <si>
+    <t>What If You Could See Your
+Future Body Right Now?
+Finally, a keto solution that works with your life, not against it. AI-powered guidance that adapts to your taste, schedule, and goals.</t>
+  </si>
+  <si>
+    <t>https://remixable.net/join/</t>
+  </si>
+  <si>
+    <t>Remixable Includes The Fastest, Simplest... &amp; Yet Most Powerful (And NEWEST!) Way To Build Pages In 2022</t>
+  </si>
+  <si>
+    <t>https://www.getkidstaleai.com/live/</t>
+  </si>
+  <si>
+    <t>Tap Into the BILLION-DOLLAR UNTAPPED GOLDMINE of Kids Story Videos!</t>
+  </si>
+  <si>
+    <t>https://microsaasai.live/microsaas-fast-pass/</t>
+  </si>
+  <si>
+    <t>How Would You Like A Fast Pass To The Funnel</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -73,6 +99,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FF2D2D2D"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="30"/>
+      <color rgb="FF0179BE"/>
+      <name val="Poppins"/>
     </font>
   </fonts>
   <fills count="2">
@@ -122,7 +160,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -131,6 +169,13 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -434,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.7109375" customWidth="1"/>
@@ -461,15 +506,71 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="186" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="57" x14ac:dyDescent="1.55">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>6</v>
       </c>
     </row>
@@ -477,7 +578,12 @@
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{3F5645DE-D60D-4810-A058-FF51F185C5D1}"/>
     <hyperlink ref="E2" r:id="rId2" xr:uid="{4A44B6D6-0773-486B-8E4C-C13673DB5957}"/>
+    <hyperlink ref="E3" r:id="rId3" xr:uid="{22AB5BC5-25AC-48B9-A6AA-FFEA11B49AD6}"/>
+    <hyperlink ref="E4" r:id="rId4" xr:uid="{875A9A5A-BCAD-4536-BC60-E363E6BBEA19}"/>
+    <hyperlink ref="E5" r:id="rId5" xr:uid="{07B8A0F4-00AE-4536-9513-22F2D01EF4EA}"/>
+    <hyperlink ref="E6" r:id="rId6" xr:uid="{B05E1D47-9839-4AF7-8B2B-0A3E1E223A14}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>